<commit_message>
fix(excel): hide TG nộp and Tổng TG trừ giờ columns in 04_CAT_LONG template
Col 6 (TG nộp) and col 8 (Tổng TG trừ giờ) are now hidden by default.
Only col 7 (TG làm thực tế) remains visible.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aa1KZAdoEWA5DLEotDGrcJ
</commit_message>
<xml_diff>
--- a/backend/templates/04_CAT_LONG_template.xlsx
+++ b/backend/templates/04_CAT_LONG_template.xlsx
@@ -793,8 +793,9 @@
     <col min="3" max="3" width="24.2857142857143" customWidth="1"/>
     <col min="4" max="4" width="15.1428571428571" customWidth="1"/>
     <col min="5" max="5" width="16.8571428571429" customWidth="1"/>
-    <col min="6" max="7" width="8.71428571428571" customWidth="1"/>
-    <col min="8" max="8" width="8.14285714285714" customWidth="1"/>
+    <col min="6" max="6" width="8.71428571428571" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="8.71428571428571" customWidth="1"/>
+    <col min="8" max="8" width="8.14285714285714" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="15.1428571428571" customWidth="1"/>
     <col min="10" max="10" width="7.85714285714286" customWidth="1"/>
     <col min="11" max="11" width="8.71428571428571" customWidth="1"/>

</xml_diff>